<commit_message>
fix: FECHA_ALTA/MODIFICA en INSERT CLIENTE; CLAVE_PAIS desde Excel; template actualizado
</commit_message>
<xml_diff>
--- a/public/template_contratos.xlsx
+++ b/public/template_contratos.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -111,6 +111,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -477,12 +480,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
@@ -515,20 +518,25 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>CLAVE_PAIS</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>CLAVE_CLIENTE</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>NOMBRE_CLIENTE</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>CLAVE_PLATAFORMA</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
@@ -545,22 +553,27 @@
           <t>Contrato Banco Ejemplo 2025</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>CLI_BANCO_EJEMPLO</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Banco Ejemplo S.A. de C.V.</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>RW6_JAVA</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Contrato inicial</t>
         </is>
@@ -568,8 +581,9 @@
     </row>
     <row r="5" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: validar reportes en inventario al subir contrato; quitar fechas estimadas de hoja REPORTES; mostrar invalidos en preview
</commit_message>
<xml_diff>
--- a/public/template_contratos.xlsx
+++ b/public/template_contratos.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -113,6 +113,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -596,10 +602,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -608,20 +614,20 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>TEMPLATE — REPORTES POR CONTRATO</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Un reporte por fila  |  CLAVE_CONTRATO debe coincidir con hoja CONTRATO  |  Fechas en formato AAAA-MM-DD</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>CLAVE_CONTRATO debe coincidir con hoja CONTRATO  |  CLAVE_REP = clave general del reporte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>CLAVE_CONTRATO</t>
@@ -632,115 +638,61 @@
           <t>CLAVE_REP</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>FECHA_ESTIMADA_QA</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>FECHA_ESTIMADA_CERT</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>FECHA_ESTIMADA_PROD</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>NOTAS</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>CONT_BANCO_EJEMPLO_01</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>MX_BM_ACLME_67</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>2025-03-01</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>2025-06-01</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>2025-09-01</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>CONT_BANCOF_2025_01</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>GT_BM_AC_AC_00</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>CONT_BANCO_EJEMPLO_01</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>MX_BM_ACLME_68</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>2025-03-01</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>2025-06-01</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>2025-09-01</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>CONT_BANCOF_2025_01</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>GT_BM_AD_AD_00</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONT_BANCO_EJEMPLO_01</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>MX_BM_R01A_0111_00_22</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>2025-04-01</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>2025-07-01</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>2025-10-01</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr"/>
-    </row>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>CONT_BANCOP_2025_01</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>MX_BM_ACLME_ACLME_01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>